<commit_message>
commit for the change for the final data straction
</commit_message>
<xml_diff>
--- a/config/patterns.xlsx
+++ b/config/patterns.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,17 +744,110 @@
           <t>Primary Concept (Column 0 - Unnamed: 0): NORMAL DATA. Secondary Concept (Column 1 - Unnamed: 1): NORMAL DATA.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Columns 3-1 (0 columns), TIME SERIES DATA</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>row-wise</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>anex-GEIH-dic2025</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GII: CO Unemployment - National, 13 Cities and Metropolitan Areas (M)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Primary Concept (Column 0 - Concepto): NORMAL DATA. Secondary Concept (Column 1 - 2001): NORMAL DATA. Third Concept (Column 2 - Unnamed: 2): NORMAL DATA.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Columns 3-300 (298 columns), TIME SERIES DATA</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>row-wise</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>anex-ELIC-SerieCoberGeo-nov2025</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>GII: AR IPP Detail</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Primary Concept (Column 0 - Años y meses): NORMAL DATA. Secondary Concept (Column 1 - Unnamed: 1): NORMAL DATA. Third Concept (Column 2 - Total): NORMAL DATA.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Columns 3-13 (11 columns), TIME SERIES DATA</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>row-wise</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sample2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>GII: AR Construction Activity</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Primary Concept (Column 0 - Unnamed: 0): NORMAL DATA. Secondary Concept (Column 1 - Unnamed: 1): NORMAL DATA.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Columns 3-1 (0 columns), TIME SERIES DATA</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>row-wise</t>
         </is>

</xml_diff>